<commit_message>
LHR-12 arrives: the Lahore set is complete at twenty
The sixteenth voice note had not downloaded. It is Bahria Town, and it was
transcribed in Hindi script when no language was forced, which is how it was
identified before being trusted.

Only that clip was transcribed, not the other nineteen again. Asking a question
about one row should cost one row.

Complete set, twenty of twenty:

  strict   30% -> 40%   gap +10 points
  spoken   75% -> 85%   gap +10 points
  WER      4.6% -> 1.9%

The gap holds at ten points under both scorings, as it did at eleven with
nineteen.

Also noted a caveat on the synthetic set: two of its clips came back in Hindi
script on the keyterms-off run only, so part of its 65% to 100% jump is a
language guess rather than the pack. The real-voice set has none of that, which
is one more reason to lead with it.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/measurement/lahore_human_manifest.xlsx
+++ b/measurement/lahore_human_manifest.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K20"/>
+  <dimension ref="A1:K21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1483,6 +1483,59 @@
       <c r="K20" t="inlineStr">
         <is>
           <t>S=0, D=0, I=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>LHR-12</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>lhr-12.ogg</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Apartment 7, Block F, Bahria Town Lahore</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Apartment 7, Block F, Bahria Town, Lahore.</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>S=0, D=0, I=0</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Apartment 7, Block F, Bahria Town, Lahore.</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>S=0, D=0, I=0</t>
         </is>
       </c>
     </row>

</xml_diff>